<commit_message>
Site_Definition_Cleanup: add GitVersion.py and patch site definition xlsx files
- src/GitVersion.py: new module exposing MAES version and git metadata
  (MAES_VERSION, GIT_DESCRIBE, GIT_BRANCH, GIT_COMMIT) with graceful
  degradation if git is unavailable; callable as a CLI diagnostic
- Patch all site definition xlsx files in C3_Prototypical_Sites, MEET2,
  and TrainingExamples: add Operator and Prototypical Site Number columns
  to Facilities tab, append maesVersion/gitDescribe to Global Simulation
  Parameters, and rename columns updated in model definitions
  (Inlet Flow At Max Primary Flow → Tank Inlet Flow at Max Downstream
  Equipment Capacity; Max Primary Outlet Flow → Max Downstream Equipment
  Capacity; Crankcase to Exhaust Emissions → CCEE Ratio Distribution)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input/Studies/MEET2/ConstantSeparator.xlsx
+++ b/input/Studies/MEET2/ConstantSeparator.xlsx
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -607,6 +607,30 @@
       <c r="B6" t="inlineStr">
         <is>
           <t>Common</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>maesVersion</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0.4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>gitDescribe</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>v0.2.0-185-g1ee2031-dirty</t>
         </is>
       </c>
     </row>
@@ -806,7 +830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -842,6 +866,16 @@
           <t>Model ID</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Prototypical Site Number</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -863,16 +897,46 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>Facility.json</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>MAES</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>MAES</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="5" t="n"/>
       <c r="C3" s="5" t="n"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>MAES</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>MAES</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="B4" s="5" t="n"/>
       <c r="C4" s="5" t="n"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>MAES</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>MAES</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2041,10 +2105,6 @@
           <t>FFDumpService.json</t>
         </is>
       </c>
-      <c r="B2">
-        <f>"FFDump"&amp;C2</f>
-        <v/>
-      </c>
       <c r="C2" t="n">
         <v>500</v>
       </c>
@@ -2055,10 +2115,6 @@
           <t>FFDumpService.json</t>
         </is>
       </c>
-      <c r="B3">
-        <f>"FFDump"&amp;C3</f>
-        <v/>
-      </c>
       <c r="C3" t="n">
         <v>600</v>
       </c>
@@ -2069,10 +2125,6 @@
           <t>FFDumpService.json</t>
         </is>
       </c>
-      <c r="B4">
-        <f>"FFDump"&amp;C4</f>
-        <v/>
-      </c>
       <c r="C4" t="n">
         <v>601</v>
       </c>
@@ -2082,10 +2134,6 @@
         <is>
           <t>FFDumpService.json</t>
         </is>
-      </c>
-      <c r="B5">
-        <f>"FFDump"&amp;C5</f>
-        <v/>
       </c>
       <c r="C5" t="n">
         <v>590</v>

</xml_diff>

<commit_message>
ConstantSeparator: replace DumpID formulas with static values
Formula '="FFDump"&C2' result cache was never populated in the repo copy,
causing Pass C blank-value errors when read programmatically. Replaced with
static values FFDump500, FFDump600, FFDump601, FFDump590.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input/Studies/MEET2/ConstantSeparator.xlsx
+++ b/input/Studies/MEET2/ConstantSeparator.xlsx
@@ -2105,6 +2105,11 @@
           <t>FFDumpService.json</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>FFDump500</t>
+        </is>
+      </c>
       <c r="C2" t="n">
         <v>500</v>
       </c>
@@ -2115,6 +2120,11 @@
           <t>FFDumpService.json</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>FFDump600</t>
+        </is>
+      </c>
       <c r="C3" t="n">
         <v>600</v>
       </c>
@@ -2125,6 +2135,11 @@
           <t>FFDumpService.json</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>FFDump601</t>
+        </is>
+      </c>
       <c r="C4" t="n">
         <v>601</v>
       </c>
@@ -2133,6 +2148,11 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>FFDumpService.json</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>FFDump590</t>
         </is>
       </c>
       <c r="C5" t="n">

</xml_diff>